<commit_message>
feat: add tea party SVG sample to Alice (DEV-6536)
Adds Tenniel's Mad Tea Party illustration as a vector graphic so that
Alice covers every supported media type now that StillImageSVGFileValue
support has shipped (see DEV-5966, DEV-6093, project "Support SVG
Vector Graphics").

- New resource I_104 (:ImageOriginal) referencing
  data/multimedia/image/IMG_teaparty_tenniel.svg
- Source: Wikimedia Commons, File:Teaparty.svg, John Tenniel, 1865,
  Public Domain Mark 1.0
- Linked to characters CH_001 (Alice), CH_004 (Hatter), CH_007 (Dormouse),
  CH_018 (March Hare); Story ST_001
- Verified via dsp-tools start-stack + create + xmlupload on localhost;
  resource renders in dsp-app's OSD viewer

Note: regen also touched non-Image CSVs (Audio, Material, etc.) where
file-size values were dropped. Out of scope for this PR; to be triaged
separately (likely a regression in xmllib's file-size handling).

Closes DEV-6536
</commit_message>
<xml_diff>
--- a/data/raw/Image.xlsx
+++ b/data/raw/Image.xlsx
@@ -377,7 +377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O104"/>
+  <dimension ref="A1:O105"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.42578125" defaultRowHeight="19"/>
   <cols>
     <col width="5.5703125" customWidth="1" style="8" min="1" max="1"/>
@@ -7689,6 +7689,66 @@
       <c r="O104" s="13" t="inlineStr">
         <is>
           <t>image_alternative</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>I_104</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>IMG_teaparty_tenniel.svg</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Public Domain</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Public Domain</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>John Tenniel</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Mad Tea Party scene by Tenniel from the 1865 first edition</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>ST_001</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>CH_001, CH_004, CH_007, CH_018</t>
+        </is>
+      </c>
+      <c r="K105" t="n">
+        <v>104</v>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>Noémi Villars-Amberg, Daniela Subotic</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>image</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add tea party SVG sample to Alice (DEV-6536) (#111)
Co-authored-by: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/Image.xlsx
+++ b/data/raw/Image.xlsx
@@ -377,7 +377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O104"/>
+  <dimension ref="A1:O105"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.42578125" defaultRowHeight="19"/>
   <cols>
     <col width="5.5703125" customWidth="1" style="8" min="1" max="1"/>
@@ -7689,6 +7689,66 @@
       <c r="O104" s="13" t="inlineStr">
         <is>
           <t>image_alternative</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>I_104</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>IMG_teaparty_tenniel.svg</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Public Domain</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Public Domain</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>John Tenniel</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Mad Tea Party scene by Tenniel from the 1865 first edition</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>ST_001</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>CH_001, CH_004, CH_007, CH_018</t>
+        </is>
+      </c>
+      <c r="K105" t="n">
+        <v>104</v>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>Noémi Villars-Amberg, Daniela Subotic</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>image</t>
         </is>
       </c>
     </row>

</xml_diff>